<commit_message>
Auto commit at 2026-03-04 14:44:25.64
</commit_message>
<xml_diff>
--- a/data/homepage.xlsx
+++ b/data/homepage.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="5" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" codeName="ThisWorkbook" defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" activeTab="5"/>
+    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" activeTab="7"/>
   </bookViews>
   <sheets>
     <sheet name="Metrics" sheetId="1" r:id="rId1"/>
@@ -1285,7 +1285,7 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="43" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="176" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -1318,6 +1318,12 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="46">
@@ -1696,7 +1702,7 @@
         <v>25</v>
       </c>
       <c r="B2" s="1">
-        <v>291041.245</v>
+        <v>45750.64</v>
       </c>
       <c r="C2" t="s">
         <v>1</v>
@@ -1708,7 +1714,7 @@
         <v>26</v>
       </c>
       <c r="B3" s="1">
-        <v>266793.69999999995</v>
+        <v>39332.979999999996</v>
       </c>
       <c r="C3" t="s">
         <v>3</v>
@@ -1720,7 +1726,7 @@
         <v>27</v>
       </c>
       <c r="B4" s="1">
-        <v>100815.54000000001</v>
+        <v>15678.32</v>
       </c>
       <c r="C4" t="s">
         <v>3</v>
@@ -1732,7 +1738,7 @@
         <v>28</v>
       </c>
       <c r="B5" s="2">
-        <v>11553</v>
+        <v>1847</v>
       </c>
       <c r="C5" t="s">
         <v>5</v>
@@ -1744,7 +1750,7 @@
         <v>29</v>
       </c>
       <c r="B6" s="1">
-        <v>871677.01500000001</v>
+        <v>971202.56000000006</v>
       </c>
       <c r="C6" t="s">
         <v>0</v>
@@ -1755,7 +1761,7 @@
         <v>30</v>
       </c>
       <c r="B7" s="1">
-        <v>719588.15</v>
+        <v>808258.14</v>
       </c>
       <c r="C7" t="s">
         <v>2</v>
@@ -1766,7 +1772,7 @@
         <v>31</v>
       </c>
       <c r="B8" s="1">
-        <v>265250.09999999998</v>
+        <v>299594.69</v>
       </c>
       <c r="C8" t="s">
         <v>2</v>
@@ -1777,7 +1783,7 @@
         <v>32</v>
       </c>
       <c r="B9" s="2">
-        <v>35029</v>
+        <v>39022</v>
       </c>
       <c r="C9" t="s">
         <v>4</v>
@@ -1788,7 +1794,7 @@
         <v>33</v>
       </c>
       <c r="B10" s="1">
-        <v>34972928.735000007</v>
+        <v>35072454.289999999</v>
       </c>
       <c r="C10" t="s">
         <v>0</v>
@@ -1800,7 +1806,7 @@
         <v>34</v>
       </c>
       <c r="B11" s="1">
-        <v>32765580.939999998</v>
+        <v>32854250.93</v>
       </c>
       <c r="C11" t="s">
         <v>2</v>
@@ -1812,7 +1818,7 @@
         <v>35</v>
       </c>
       <c r="B12" s="1">
-        <v>12211063.960000001</v>
+        <v>12245408.550000001</v>
       </c>
       <c r="C12" t="s">
         <v>2</v>
@@ -1823,7 +1829,7 @@
         <v>36</v>
       </c>
       <c r="B13" s="2">
-        <v>1352936</v>
+        <v>1356929</v>
       </c>
       <c r="C13" t="s">
         <v>4</v>
@@ -1907,6 +1913,14 @@
     <row r="3" spans="1:3" x14ac:dyDescent="0.15">
       <c r="A3" t="s">
         <v>10</v>
+      </c>
+      <c r="B3">
+        <f>255055.85+89760.3</f>
+        <v>344816.15</v>
+      </c>
+      <c r="C3">
+        <f>94835.53+24646.28</f>
+        <v>119481.81</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.15">
@@ -3935,8 +3949,27 @@
       </c>
     </row>
     <row r="94" spans="1:6" x14ac:dyDescent="0.15">
-      <c r="D94" s="4"/>
-      <c r="E94" s="4"/>
+      <c r="A94" s="17">
+        <v>46055</v>
+      </c>
+      <c r="B94" s="18">
+        <v>344816.15</v>
+      </c>
+      <c r="C94" s="18">
+        <f>57206.52+139442.38</f>
+        <v>196648.9</v>
+      </c>
+      <c r="D94" s="19">
+        <v>119481.81</v>
+      </c>
+      <c r="E94" s="19">
+        <f>D94+C94</f>
+        <v>316130.70999999996</v>
+      </c>
+      <c r="F94" s="18">
+        <f>10561+3138</f>
+        <v>13699</v>
+      </c>
     </row>
     <row r="95" spans="1:6" x14ac:dyDescent="0.15">
       <c r="D95" s="14"/>
@@ -3951,7 +3984,7 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Sheet6"/>
-  <dimension ref="A1:K90"/>
+  <dimension ref="A1:K92"/>
   <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="12" max="12" width="19.25" customWidth="1"/>
@@ -7107,6 +7140,43 @@
       <c r="K90" s="10">
         <v>10040</v>
       </c>
+    </row>
+    <row r="91" spans="1:11" x14ac:dyDescent="0.15">
+      <c r="A91" s="9">
+        <v>46055</v>
+      </c>
+      <c r="B91" s="16">
+        <v>6497.78</v>
+      </c>
+      <c r="C91" s="16">
+        <v>2174.98</v>
+      </c>
+      <c r="D91" s="16">
+        <v>7166.2</v>
+      </c>
+      <c r="E91" s="16">
+        <v>2564.1</v>
+      </c>
+      <c r="F91" s="10">
+        <v>1515</v>
+      </c>
+      <c r="G91" s="10"/>
+      <c r="H91" s="10"/>
+      <c r="I91" s="10">
+        <v>8265</v>
+      </c>
+      <c r="J91" s="10"/>
+      <c r="K91" s="10">
+        <v>8750</v>
+      </c>
+    </row>
+    <row r="92" spans="1:11" x14ac:dyDescent="0.15">
+      <c r="F92" s="20"/>
+      <c r="G92" s="20"/>
+      <c r="H92" s="20"/>
+      <c r="I92" s="20"/>
+      <c r="J92" s="20"/>
+      <c r="K92" s="20"/>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
@@ -7142,6 +7212,9 @@
     <row r="3" spans="1:2" x14ac:dyDescent="0.15">
       <c r="A3" t="s">
         <v>10</v>
+      </c>
+      <c r="B3">
+        <v>36933.06</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.15">
@@ -7225,7 +7298,7 @@
     <row r="1" spans="1:15" x14ac:dyDescent="0.15">
       <c r="A1" s="3">
         <f ca="1">TODAY()-1</f>
-        <v>46077</v>
+        <v>46084</v>
       </c>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.15">
@@ -7240,7 +7313,10 @@
       <c r="A3" t="s">
         <v>42</v>
       </c>
-      <c r="B3" s="4"/>
+      <c r="B3" s="4">
+        <f>33066.49+12684.15</f>
+        <v>45750.64</v>
+      </c>
       <c r="C3" t="s">
         <v>0</v>
       </c>
@@ -7249,7 +7325,10 @@
       <c r="A4" t="s">
         <v>43</v>
       </c>
-      <c r="B4" s="4"/>
+      <c r="B4" s="4">
+        <f>28217.32+11115.66</f>
+        <v>39332.979999999996</v>
+      </c>
       <c r="C4" t="s">
         <v>2</v>
       </c>
@@ -7258,7 +7337,10 @@
       <c r="A5" t="s">
         <v>44</v>
       </c>
-      <c r="B5" s="4"/>
+      <c r="B5" s="4">
+        <f>12286.76+3391.56</f>
+        <v>15678.32</v>
+      </c>
       <c r="C5" t="s">
         <v>2</v>
       </c>
@@ -7267,7 +7349,10 @@
       <c r="A6" t="s">
         <v>45</v>
       </c>
-      <c r="B6" s="4"/>
+      <c r="B6" s="4">
+        <f>1379+468</f>
+        <v>1847</v>
+      </c>
       <c r="C6" t="s">
         <v>4</v>
       </c>
@@ -7300,18 +7385,18 @@
       </c>
       <c r="B11" s="4">
         <f>Metrics!B2</f>
-        <v>291041.245</v>
+        <v>45750.64</v>
       </c>
       <c r="C11" t="s">
         <v>0</v>
       </c>
       <c r="E11" s="5">
         <f>B11</f>
-        <v>291041.245</v>
+        <v>45750.64</v>
       </c>
       <c r="F11" s="5">
         <f>E11+B3</f>
-        <v>291041.245</v>
+        <v>91501.28</v>
       </c>
       <c r="H11" s="5"/>
       <c r="I11" s="5"/>
@@ -7324,18 +7409,18 @@
       </c>
       <c r="B12" s="4">
         <f>Metrics!B3</f>
-        <v>266793.69999999995</v>
+        <v>39332.979999999996</v>
       </c>
       <c r="C12" t="s">
         <v>2</v>
       </c>
       <c r="E12" s="5">
         <f t="shared" ref="E12:E14" si="0">B12</f>
-        <v>266793.69999999995</v>
+        <v>39332.979999999996</v>
       </c>
       <c r="F12" s="5">
         <f t="shared" ref="F12:F14" si="1">E12+B4</f>
-        <v>266793.69999999995</v>
+        <v>78665.959999999992</v>
       </c>
       <c r="H12" s="5"/>
       <c r="I12" s="5"/>
@@ -7346,18 +7431,18 @@
       </c>
       <c r="B13" s="4">
         <f>Metrics!B4</f>
-        <v>100815.54000000001</v>
+        <v>15678.32</v>
       </c>
       <c r="C13" t="s">
         <v>2</v>
       </c>
       <c r="E13" s="5">
         <f t="shared" si="0"/>
-        <v>100815.54000000001</v>
+        <v>15678.32</v>
       </c>
       <c r="F13" s="5">
         <f t="shared" si="1"/>
-        <v>100815.54000000001</v>
+        <v>31356.639999999999</v>
       </c>
       <c r="H13" s="5"/>
       <c r="I13" s="5"/>
@@ -7369,18 +7454,18 @@
       </c>
       <c r="B14" s="4">
         <f>Metrics!B5</f>
-        <v>11553</v>
+        <v>1847</v>
       </c>
       <c r="C14" t="s">
         <v>4</v>
       </c>
       <c r="E14" s="5">
         <f t="shared" si="0"/>
-        <v>11553</v>
+        <v>1847</v>
       </c>
       <c r="F14" s="5">
         <f t="shared" si="1"/>
-        <v>11553</v>
+        <v>3694</v>
       </c>
       <c r="H14" s="5"/>
       <c r="I14" s="5"/>
@@ -7392,18 +7477,18 @@
       </c>
       <c r="B15" s="4">
         <f>Metrics!B6</f>
-        <v>871677.01500000001</v>
+        <v>971202.56000000006</v>
       </c>
       <c r="C15" t="s">
         <v>0</v>
       </c>
       <c r="E15" s="5">
         <f t="shared" ref="E15:E22" si="2">B15</f>
-        <v>871677.01500000001</v>
+        <v>971202.56000000006</v>
       </c>
       <c r="F15" s="5">
         <f>E15+B3</f>
-        <v>871677.01500000001</v>
+        <v>1016953.2000000001</v>
       </c>
       <c r="G15" s="5"/>
       <c r="I15" s="5"/>
@@ -7415,18 +7500,18 @@
       </c>
       <c r="B16" s="4">
         <f>Metrics!B7</f>
-        <v>719588.15</v>
+        <v>808258.14</v>
       </c>
       <c r="C16" t="s">
         <v>2</v>
       </c>
       <c r="E16" s="5">
         <f t="shared" si="2"/>
-        <v>719588.15</v>
+        <v>808258.14</v>
       </c>
       <c r="F16" s="5">
         <f>E16+B4</f>
-        <v>719588.15</v>
+        <v>847591.12</v>
       </c>
       <c r="I16" s="5"/>
     </row>
@@ -7436,18 +7521,18 @@
       </c>
       <c r="B17" s="4">
         <f>Metrics!B8</f>
-        <v>265250.09999999998</v>
+        <v>299594.69</v>
       </c>
       <c r="C17" t="s">
         <v>2</v>
       </c>
       <c r="E17" s="5">
         <f t="shared" si="2"/>
-        <v>265250.09999999998</v>
+        <v>299594.69</v>
       </c>
       <c r="F17" s="5">
         <f t="shared" ref="F17" si="3">E17+B5</f>
-        <v>265250.09999999998</v>
+        <v>315273.01</v>
       </c>
       <c r="I17" s="5"/>
     </row>
@@ -7457,18 +7542,18 @@
       </c>
       <c r="B18" s="4">
         <f>Metrics!B9</f>
-        <v>35029</v>
+        <v>39022</v>
       </c>
       <c r="C18" t="s">
         <v>4</v>
       </c>
       <c r="E18" s="5">
         <f t="shared" si="2"/>
-        <v>35029</v>
+        <v>39022</v>
       </c>
       <c r="F18" s="5">
         <f>E18+B6</f>
-        <v>35029</v>
+        <v>40869</v>
       </c>
       <c r="H18" s="12"/>
       <c r="I18" s="5"/>
@@ -7479,18 +7564,18 @@
       </c>
       <c r="B19" s="4">
         <f>Metrics!B10</f>
-        <v>34972928.735000007</v>
+        <v>35072454.289999999</v>
       </c>
       <c r="C19" t="s">
         <v>0</v>
       </c>
       <c r="E19" s="5">
         <f>B19</f>
-        <v>34972928.735000007</v>
+        <v>35072454.289999999</v>
       </c>
       <c r="F19" s="5">
         <f>E19+B3</f>
-        <v>34972928.735000007</v>
+        <v>35118204.93</v>
       </c>
       <c r="I19" s="5"/>
       <c r="J19" s="5"/>
@@ -7501,18 +7586,18 @@
       </c>
       <c r="B20" s="4">
         <f>Metrics!B11</f>
-        <v>32765580.939999998</v>
+        <v>32854250.93</v>
       </c>
       <c r="C20" t="s">
         <v>2</v>
       </c>
       <c r="E20" s="5">
         <f t="shared" si="2"/>
-        <v>32765580.939999998</v>
+        <v>32854250.93</v>
       </c>
       <c r="F20" s="5">
         <f t="shared" ref="F20:F22" si="4">E20+B4</f>
-        <v>32765580.939999998</v>
+        <v>32893583.91</v>
       </c>
       <c r="I20" s="5"/>
       <c r="J20" s="5"/>
@@ -7523,18 +7608,18 @@
       </c>
       <c r="B21" s="4">
         <f>Metrics!B12</f>
-        <v>12211063.960000001</v>
+        <v>12245408.550000001</v>
       </c>
       <c r="C21" t="s">
         <v>2</v>
       </c>
       <c r="E21" s="5">
         <f t="shared" si="2"/>
-        <v>12211063.960000001</v>
+        <v>12245408.550000001</v>
       </c>
       <c r="F21" s="5">
         <f t="shared" si="4"/>
-        <v>12211063.960000001</v>
+        <v>12261086.870000001</v>
       </c>
       <c r="I21" s="5"/>
       <c r="J21" s="5"/>
@@ -7545,18 +7630,18 @@
       </c>
       <c r="B22" s="4">
         <f>Metrics!B13</f>
-        <v>1352936</v>
+        <v>1356929</v>
       </c>
       <c r="C22" t="s">
         <v>4</v>
       </c>
       <c r="E22" s="5">
         <f t="shared" si="2"/>
-        <v>1352936</v>
+        <v>1356929</v>
       </c>
       <c r="F22" s="5">
         <f t="shared" si="4"/>
-        <v>1352936</v>
+        <v>1358776</v>
       </c>
       <c r="H22" s="12"/>
       <c r="I22" s="5"/>
@@ -7739,10 +7824,12 @@
         <v>191</v>
       </c>
       <c r="B10" s="4">
-        <v>580496.03</v>
+        <f>580496.03+344816.15</f>
+        <v>925312.18</v>
       </c>
       <c r="C10" s="5">
-        <v>164409.51999999999</v>
+        <f>164409.52+119481.81</f>
+        <v>283891.32999999996</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.15">
@@ -7842,7 +7929,7 @@
         <v>2026</v>
       </c>
       <c r="B10" s="5">
-        <v>48807.1</v>
+        <v>85471.13</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.15">

</xml_diff>

<commit_message>
Auto commit at 2026-04-03 16:02:19.07
</commit_message>
<xml_diff>
--- a/data/homepage.xlsx
+++ b/data/homepage.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" codeName="ThisWorkbook" defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010"/>
+    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" activeTab="8"/>
   </bookViews>
   <sheets>
     <sheet name="Metrics" sheetId="1" r:id="rId1"/>
@@ -1323,10 +1323,10 @@
     <xf numFmtId="4" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="181" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="181" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="46">
     <cellStyle name="20% - 着色 1" xfId="17" builtinId="30" customBuiltin="1"/>
@@ -1929,6 +1929,12 @@
       <c r="A4" t="s">
         <v>11</v>
       </c>
+      <c r="B4">
+        <v>450668.16</v>
+      </c>
+      <c r="C4">
+        <v>154708.91</v>
+      </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.15">
       <c r="A5" t="s">
@@ -1990,7 +1996,7 @@
     <col min="1" max="1" width="17.125" style="6" customWidth="1"/>
     <col min="2" max="2" width="17.125" customWidth="1"/>
     <col min="3" max="3" width="19.375" customWidth="1"/>
-    <col min="4" max="4" width="16.5" customWidth="1"/>
+    <col min="4" max="4" width="22.75" customWidth="1"/>
     <col min="5" max="5" width="20.875" customWidth="1"/>
     <col min="6" max="6" width="14.5" customWidth="1"/>
     <col min="10" max="10" width="24.25" customWidth="1"/>
@@ -3974,8 +3980,24 @@
       </c>
     </row>
     <row r="95" spans="1:6" x14ac:dyDescent="0.15">
-      <c r="D95" s="14"/>
-      <c r="E95" s="14"/>
+      <c r="A95" s="17">
+        <v>46084</v>
+      </c>
+      <c r="B95" s="10">
+        <v>450668.16</v>
+      </c>
+      <c r="C95" s="10">
+        <v>231015.32</v>
+      </c>
+      <c r="D95" s="19">
+        <v>154708.91</v>
+      </c>
+      <c r="E95" s="19">
+        <v>385724.23</v>
+      </c>
+      <c r="F95" s="10">
+        <v>18788</v>
+      </c>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
@@ -7162,23 +7184,54 @@
       <c r="F91" s="10">
         <v>1515</v>
       </c>
-      <c r="G91" s="10"/>
-      <c r="H91" s="10"/>
+      <c r="G91" s="10">
+        <v>0</v>
+      </c>
+      <c r="H91" s="10">
+        <v>0</v>
+      </c>
       <c r="I91" s="10">
         <v>8265</v>
       </c>
-      <c r="J91" s="10"/>
+      <c r="J91" s="10">
+        <v>0</v>
+      </c>
       <c r="K91" s="10">
         <v>8750</v>
       </c>
     </row>
     <row r="92" spans="1:11" x14ac:dyDescent="0.15">
-      <c r="F92" s="20"/>
-      <c r="G92" s="20"/>
-      <c r="H92" s="20"/>
-      <c r="I92" s="20"/>
-      <c r="J92" s="20"/>
-      <c r="K92" s="20"/>
+      <c r="A92" s="9">
+        <v>46084</v>
+      </c>
+      <c r="B92" s="21">
+        <v>5759.6</v>
+      </c>
+      <c r="C92" s="21">
+        <v>1603.87</v>
+      </c>
+      <c r="D92" s="21">
+        <v>9252.93</v>
+      </c>
+      <c r="E92" s="21">
+        <v>2200.4</v>
+      </c>
+      <c r="F92" s="10">
+        <v>2110</v>
+      </c>
+      <c r="G92" s="10">
+        <v>0</v>
+      </c>
+      <c r="H92" s="10"/>
+      <c r="I92" s="10">
+        <v>10840</v>
+      </c>
+      <c r="J92" s="10">
+        <v>0</v>
+      </c>
+      <c r="K92" s="10">
+        <v>12740</v>
+      </c>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
@@ -7222,6 +7275,9 @@
     <row r="4" spans="1:2" x14ac:dyDescent="0.15">
       <c r="A4" t="s">
         <v>11</v>
+      </c>
+      <c r="B4">
+        <v>44506.8</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.15">
@@ -7300,7 +7356,7 @@
     <row r="1" spans="1:15" x14ac:dyDescent="0.15">
       <c r="A1" s="3">
         <f ca="1">TODAY()-1</f>
-        <v>46092</v>
+        <v>46114</v>
       </c>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.15">
@@ -7337,7 +7393,7 @@
       <c r="A5" t="s">
         <v>44</v>
       </c>
-      <c r="B5" s="21">
+      <c r="B5" s="20">
         <v>20689.639999999996</v>
       </c>
       <c r="C5" t="s">
@@ -7725,10 +7781,10 @@
         <v>64</v>
       </c>
       <c r="B2" s="4">
-        <v>626624.99</v>
+        <v>229889.73</v>
       </c>
       <c r="C2" s="5">
-        <v>419522.88</v>
+        <v>152374.23000000001</v>
       </c>
       <c r="G2" s="4"/>
     </row>
@@ -7737,10 +7793,10 @@
         <v>65</v>
       </c>
       <c r="B3" s="4">
-        <v>2487651.48</v>
+        <v>1380267.33</v>
       </c>
       <c r="C3" s="5">
-        <v>1298604.49</v>
+        <v>708782.7</v>
       </c>
       <c r="G3" s="4"/>
     </row>
@@ -7749,10 +7805,10 @@
         <v>66</v>
       </c>
       <c r="B4" s="4">
-        <v>3580420.55</v>
+        <v>2965107.6</v>
       </c>
       <c r="C4" s="5">
-        <v>1340324.3400000001</v>
+        <v>1062875.79</v>
       </c>
       <c r="G4" s="4"/>
     </row>
@@ -7761,10 +7817,10 @@
         <v>67</v>
       </c>
       <c r="B5" s="4">
-        <v>4883275.16</v>
+        <v>4260538.4800000004</v>
       </c>
       <c r="C5" s="5">
-        <v>1541074.64</v>
+        <v>1260741.8400000001</v>
       </c>
       <c r="G5" s="4"/>
     </row>
@@ -7773,10 +7829,10 @@
         <v>68</v>
       </c>
       <c r="B6" s="4">
-        <v>5136589.43</v>
+        <v>4790817.5599999996</v>
       </c>
       <c r="C6" s="5">
-        <v>2141138.69</v>
+        <v>2006748.84</v>
       </c>
       <c r="G6" s="13"/>
     </row>
@@ -7785,10 +7841,10 @@
         <v>69</v>
       </c>
       <c r="B7" s="4">
-        <v>5076097.29</v>
+        <v>4889614.41</v>
       </c>
       <c r="C7" s="5">
-        <v>1765909.85</v>
+        <v>1694937.89</v>
       </c>
       <c r="G7" s="5"/>
     </row>
@@ -7797,11 +7853,10 @@
         <v>70</v>
       </c>
       <c r="B8" s="4">
-        <f>6674722.09</f>
-        <v>6674722.0899999999</v>
+        <v>6669309.1900000004</v>
       </c>
       <c r="C8" s="5">
-        <v>1775147.16</v>
+        <v>1773151.96</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.15">
@@ -7809,12 +7864,10 @@
         <v>71</v>
       </c>
       <c r="B9" s="4">
-        <f>4367131.47+429127.72+43.76+406461.36-57.19+433385.02</f>
-        <v>5636092.1399999987</v>
+        <v>5635870.7300000004</v>
       </c>
       <c r="C9" s="5">
-        <f>1270602.14+136362.21+8.63+124997.05-13.15+132190.9</f>
-        <v>1664147.7799999998</v>
+        <v>1664091.82</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.15">
@@ -7822,12 +7875,10 @@
         <v>191</v>
       </c>
       <c r="B10" s="4">
-        <f>580496.03+344816.15</f>
-        <v>925312.18</v>
+        <v>1376120.09</v>
       </c>
       <c r="C10" s="5">
-        <f>164409.52+119481.81</f>
-        <v>283891.32999999996</v>
+        <v>438625.28000000003</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.15">
@@ -7927,7 +7978,7 @@
         <v>2026</v>
       </c>
       <c r="B10" s="5">
-        <v>85471.13</v>
+        <v>139072.76999999999</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.15">
@@ -8250,7 +8301,7 @@
         <v>2026</v>
       </c>
       <c r="C27">
-        <v>6354.57</v>
+        <v>18611.95</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.15">
@@ -8261,7 +8312,7 @@
         <v>2026</v>
       </c>
       <c r="C28">
-        <v>1655.3</v>
+        <v>5434.15</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.15">
@@ -8272,7 +8323,7 @@
         <v>2026</v>
       </c>
       <c r="C29">
-        <v>2400</v>
+        <v>6025</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.15">
@@ -8283,7 +8334,7 @@
         <v>2026</v>
       </c>
       <c r="C30">
-        <v>13308</v>
+        <v>37891.9</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.15">
@@ -8294,7 +8345,8 @@
         <v>2026</v>
       </c>
       <c r="C31">
-        <v>2950.2</v>
+        <f>5764.5+1957.1</f>
+        <v>7721.6</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.15">
@@ -8316,7 +8368,7 @@
         <v>2026</v>
       </c>
       <c r="C33">
-        <v>11830</v>
+        <v>30935</v>
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.15">
@@ -8338,7 +8390,7 @@
         <v>2026</v>
       </c>
       <c r="C35">
-        <v>10040</v>
+        <v>31530</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto commit at 2026-05-01 11:02:11.23
</commit_message>
<xml_diff>
--- a/data/homepage.xlsx
+++ b/data/homepage.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" codeName="ThisWorkbook" defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" activeTab="8"/>
+    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" firstSheet="1" activeTab="8"/>
   </bookViews>
   <sheets>
     <sheet name="Metrics" sheetId="1" r:id="rId1"/>
@@ -4008,7 +4008,7 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Sheet6"/>
-  <dimension ref="A1:K92"/>
+  <dimension ref="A1:K93"/>
   <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="12" max="12" width="19.25" customWidth="1"/>
@@ -7231,6 +7231,42 @@
       </c>
       <c r="K92" s="10">
         <v>12740</v>
+      </c>
+    </row>
+    <row r="93" spans="1:11" x14ac:dyDescent="0.15">
+      <c r="A93" s="9">
+        <v>46116</v>
+      </c>
+      <c r="B93" s="10">
+        <v>5844.86</v>
+      </c>
+      <c r="C93" s="10">
+        <v>1375.75</v>
+      </c>
+      <c r="D93" s="10">
+        <v>11901</v>
+      </c>
+      <c r="E93" s="10">
+        <f>2215.9+535.9</f>
+        <v>2751.8</v>
+      </c>
+      <c r="F93" s="10">
+        <v>900</v>
+      </c>
+      <c r="G93" s="10">
+        <v>0</v>
+      </c>
+      <c r="H93" s="10">
+        <v>0</v>
+      </c>
+      <c r="I93" s="10">
+        <v>9295</v>
+      </c>
+      <c r="J93" s="10">
+        <v>0</v>
+      </c>
+      <c r="K93" s="10">
+        <v>10480</v>
       </c>
     </row>
   </sheetData>
@@ -7283,6 +7319,9 @@
     <row r="5" spans="1:2" x14ac:dyDescent="0.15">
       <c r="A5" t="s">
         <v>12</v>
+      </c>
+      <c r="B5">
+        <v>42548.41</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.15">
@@ -7356,7 +7395,7 @@
     <row r="1" spans="1:15" x14ac:dyDescent="0.15">
       <c r="A1" s="3">
         <f ca="1">TODAY()-1</f>
-        <v>46114</v>
+        <v>46142</v>
       </c>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.15">
@@ -7998,6 +8037,7 @@
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
     <col min="3" max="3" width="12.125" customWidth="1"/>
+    <col min="5" max="5" width="13.625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.15">
@@ -8301,7 +8341,8 @@
         <v>2026</v>
       </c>
       <c r="C27">
-        <v>18611.95</v>
+        <f>18611.95+5844.86</f>
+        <v>24456.81</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.15">
@@ -8312,7 +8353,8 @@
         <v>2026</v>
       </c>
       <c r="C28">
-        <v>5434.15</v>
+        <f>5434.15+1375.75</f>
+        <v>6809.9</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.15">
@@ -8323,7 +8365,8 @@
         <v>2026</v>
       </c>
       <c r="C29">
-        <v>6025</v>
+        <f>6025+900</f>
+        <v>6925</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.15">
@@ -8334,7 +8377,8 @@
         <v>2026</v>
       </c>
       <c r="C30">
-        <v>37891.9</v>
+        <f>37891.9+11901</f>
+        <v>49792.9</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.15">
@@ -8345,8 +8389,8 @@
         <v>2026</v>
       </c>
       <c r="C31">
-        <f>5764.5+1957.1</f>
-        <v>7721.6</v>
+        <f>5764.5+1957.1+2751.8</f>
+        <v>10473.400000000001</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.15">
@@ -8368,7 +8412,8 @@
         <v>2026</v>
       </c>
       <c r="C33">
-        <v>30935</v>
+        <f>30935+9295</f>
+        <v>40230</v>
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.15">
@@ -8390,7 +8435,8 @@
         <v>2026</v>
       </c>
       <c r="C35">
-        <v>31530</v>
+        <f>31530+10480</f>
+        <v>42010</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto commit at 2026-05-01 12:32:10.46
</commit_message>
<xml_diff>
--- a/data/homepage.xlsx
+++ b/data/homepage.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" codeName="ThisWorkbook" defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" firstSheet="1" activeTab="8"/>
+    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" firstSheet="1" activeTab="6"/>
   </bookViews>
   <sheets>
     <sheet name="Metrics" sheetId="1" r:id="rId1"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="259" uniqueCount="192">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="258" uniqueCount="191">
   <si>
     <t>kwh</t>
   </si>
@@ -282,10 +282,6 @@
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
-    <t>充电服务费收入(元)</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
     <t>年份</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
@@ -656,7 +652,7 @@
     <t>月租车</t>
   </si>
   <si>
-    <t>2026年</t>
+    <t>充电服务费(元)</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
@@ -2004,27 +2000,27 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A1" s="7" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B1" s="8" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="C1" s="8" t="s">
+        <v>86</v>
+      </c>
+      <c r="D1" s="8" t="s">
         <v>87</v>
       </c>
-      <c r="D1" s="8" t="s">
-        <v>88</v>
-      </c>
       <c r="E1" s="8" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="F1" s="8" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A2" s="7" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="B2" s="8">
         <v>276.08</v>
@@ -2044,7 +2040,7 @@
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A3" s="7" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="B3" s="8">
         <v>60171.720000000074</v>
@@ -2064,7 +2060,7 @@
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A4" s="7" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="B4" s="8">
         <v>61781.849999999962</v>
@@ -2084,7 +2080,7 @@
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A5" s="7" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B5" s="8">
         <v>94676.269999999713</v>
@@ -2105,7 +2101,7 @@
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A6" s="7" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B6" s="8">
         <v>120954.96999999981</v>
@@ -2126,7 +2122,7 @@
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A7" s="7" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B7" s="8">
         <v>133453.96999999997</v>
@@ -2147,7 +2143,7 @@
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A8" s="7" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B8" s="8">
         <v>155310.13000000009</v>
@@ -2168,7 +2164,7 @@
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A9" s="7" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B9" s="8">
         <v>140296.57000000015</v>
@@ -2189,7 +2185,7 @@
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A10" s="7" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B10" s="8">
         <v>90221.229999999938</v>
@@ -2210,7 +2206,7 @@
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A11" s="7" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="B11" s="8">
         <v>128259.44000000009</v>
@@ -2231,7 +2227,7 @@
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A12" s="7" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B12" s="8">
         <v>186518.22000000032</v>
@@ -2252,7 +2248,7 @@
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A13" s="7" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B13" s="8">
         <v>208195.52000000005</v>
@@ -2273,7 +2269,7 @@
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A14" s="7" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B14" s="8">
         <v>207321.07999999955</v>
@@ -2294,7 +2290,7 @@
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A15" s="7" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B15" s="8">
         <v>223550.75999999975</v>
@@ -2315,7 +2311,7 @@
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A16" s="7" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B16" s="8">
         <v>223592.69999999914</v>
@@ -2336,7 +2332,7 @@
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A17" s="7" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B17" s="8">
         <v>188241.87999999995</v>
@@ -2357,7 +2353,7 @@
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A18" s="7" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B18" s="8">
         <v>238037.90999999945</v>
@@ -2378,7 +2374,7 @@
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A19" s="7" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B19" s="8">
         <v>291934.49999999901</v>
@@ -2399,7 +2395,7 @@
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A20" s="7" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B20" s="8">
         <v>361481.67000000097</v>
@@ -2420,7 +2416,7 @@
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A21" s="7" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B21" s="8">
         <f>324029.82</f>
@@ -2444,7 +2440,7 @@
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A22" s="7" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B22" s="8">
         <v>71232.629999999903</v>
@@ -2465,7 +2461,7 @@
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A23" s="7" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="B23" s="8">
         <v>171210.18</v>
@@ -2486,7 +2482,7 @@
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A24" s="7" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="B24" s="8">
         <v>221773.39000000004</v>
@@ -2507,7 +2503,7 @@
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A25" s="7" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B25" s="8">
         <v>209015.27000000031</v>
@@ -2528,7 +2524,7 @@
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A26" s="7" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="B26" s="8">
         <v>266563.71000000072</v>
@@ -2549,7 +2545,7 @@
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A27" s="7" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B27" s="8">
         <v>277446.12999999971</v>
@@ -2570,7 +2566,7 @@
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A28" s="7" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B28" s="8">
         <v>388725.31999999826</v>
@@ -2591,7 +2587,7 @@
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A29" s="7" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B29" s="8">
         <v>327347.20000000013</v>
@@ -2612,7 +2608,7 @@
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A30" s="7" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B30" s="8">
         <v>337917.21000000183</v>
@@ -2633,7 +2629,7 @@
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A31" s="7" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="B31" s="8">
         <v>416971.15000000142</v>
@@ -2654,7 +2650,7 @@
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A32" s="7" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B32" s="8">
         <v>568188.53900000243</v>
@@ -2675,7 +2671,7 @@
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A33" s="7" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B33" s="8">
         <f>538319.98+57.2</f>
@@ -2699,7 +2695,7 @@
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A34" s="7" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B34" s="8">
         <v>350926.49400000152</v>
@@ -2720,7 +2716,7 @@
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A35" s="7" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="B35" s="8">
         <v>353745.77899999841</v>
@@ -2741,7 +2737,7 @@
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A36" s="7" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="B36" s="8">
         <v>284140.44400000083</v>
@@ -2762,7 +2758,7 @@
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A37" s="7" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B37" s="8">
         <v>329970.87800000008</v>
@@ -2783,7 +2779,7 @@
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A38" s="7" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="B38" s="8">
         <v>521034.7840000001</v>
@@ -2804,7 +2800,7 @@
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A39" s="7" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="B39" s="8">
         <v>667085.79699999967</v>
@@ -2825,7 +2821,7 @@
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A40" s="7" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="B40" s="8">
         <v>370120.30400000105</v>
@@ -2846,7 +2842,7 @@
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A41" s="7" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="B41" s="8">
         <v>390662.89099999919</v>
@@ -2867,7 +2863,7 @@
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A42" s="7" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="B42" s="8">
         <v>328815.68100000039</v>
@@ -2888,7 +2884,7 @@
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A43" s="7" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B43" s="8">
         <v>328662.25099999987</v>
@@ -2909,7 +2905,7 @@
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A44" s="7" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="B44" s="8">
         <v>419732.66699999961</v>
@@ -2930,7 +2926,7 @@
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A45" s="7" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="B45" s="8">
         <v>466563.12699999998</v>
@@ -2951,7 +2947,7 @@
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A46" s="7" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B46" s="8">
         <v>369842.09899999981</v>
@@ -2972,7 +2968,7 @@
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A47" s="7" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="B47" s="8">
         <v>390410.73700000125</v>
@@ -2993,7 +2989,7 @@
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A48" s="7" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B48" s="8">
         <v>384633.24399999896</v>
@@ -3014,7 +3010,7 @@
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A49" s="7" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="B49" s="8">
         <v>432236.52799999912</v>
@@ -3035,7 +3031,7 @@
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A50" s="7" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B50" s="8">
         <v>480696.82300000201</v>
@@ -3056,7 +3052,7 @@
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A51" s="7" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B51" s="8">
         <v>540693.31500000332</v>
@@ -3077,7 +3073,7 @@
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A52" s="7" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B52" s="8">
         <v>550673.11999999988</v>
@@ -3098,7 +3094,7 @@
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A53" s="7" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="B53" s="8">
         <v>416275.09300000145</v>
@@ -3119,7 +3115,7 @@
     </row>
     <row r="54" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A54" s="7" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="B54" s="8">
         <v>373518.10800000158</v>
@@ -3140,7 +3136,7 @@
     </row>
     <row r="55" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A55" s="7" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="B55" s="8">
         <v>367617.62999999966</v>
@@ -3161,7 +3157,7 @@
     </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A56" s="7" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="B56" s="8">
         <v>363429.61099999945</v>
@@ -3182,7 +3178,7 @@
     </row>
     <row r="57" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A57" s="7" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="B57" s="8">
         <v>308208.74899999989</v>
@@ -3203,7 +3199,7 @@
     </row>
     <row r="58" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A58" s="7" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="B58" s="8">
         <v>421405.62000000081</v>
@@ -3224,7 +3220,7 @@
     </row>
     <row r="59" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A59" s="7" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="B59" s="8">
         <v>449170.92499999941</v>
@@ -3245,7 +3241,7 @@
     </row>
     <row r="60" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A60" s="7" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="B60" s="8">
         <v>431602.59000000008</v>
@@ -3266,7 +3262,7 @@
     </row>
     <row r="61" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A61" s="7" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="B61" s="8">
         <v>432741.64299999847</v>
@@ -3287,7 +3283,7 @@
     </row>
     <row r="62" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A62" s="7" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="B62" s="8">
         <v>430446.36099999736</v>
@@ -3308,7 +3304,7 @@
     </row>
     <row r="63" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A63" s="7" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="B63" s="8">
         <v>500972.23800000071</v>
@@ -3329,7 +3325,7 @@
     </row>
     <row r="64" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A64" s="7" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="B64" s="8">
         <v>489071.34400000138</v>
@@ -3350,7 +3346,7 @@
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A65" s="7" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="B65" s="8">
         <v>395557.42599999788</v>
@@ -3371,7 +3367,7 @@
     </row>
     <row r="66" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A66" s="7" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="B66" s="8">
         <v>359924.54199999914</v>
@@ -3392,7 +3388,7 @@
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A67" s="7" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="B67" s="8">
         <v>401043.42400000076</v>
@@ -3413,7 +3409,7 @@
     </row>
     <row r="68" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A68" s="7" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="B68" s="8">
         <v>455952.43099999928</v>
@@ -3434,7 +3430,7 @@
     </row>
     <row r="69" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A69" s="7" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="B69" s="8">
         <v>518763.45200000372</v>
@@ -3455,7 +3451,7 @@
     </row>
     <row r="70" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A70" s="7" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="B70" s="8">
         <v>436247.67099999828</v>
@@ -3476,7 +3472,7 @@
     </row>
     <row r="71" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A71" s="7" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="B71" s="8">
         <v>577922.50300000468</v>
@@ -3497,7 +3493,7 @@
     </row>
     <row r="72" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A72" s="7" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="B72" s="8">
         <v>522200.26800000382</v>
@@ -3518,7 +3514,7 @@
     </row>
     <row r="73" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A73" s="7" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="B73" s="8">
         <v>568926.92999999947</v>
@@ -3539,7 +3535,7 @@
     </row>
     <row r="74" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A74" s="7" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="B74" s="8">
         <v>557739.85900000052</v>
@@ -3560,7 +3556,7 @@
     </row>
     <row r="75" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A75" s="7" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="B75" s="8">
         <v>704038.67900000501</v>
@@ -3581,7 +3577,7 @@
     </row>
     <row r="76" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A76" s="7" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="B76" s="8">
         <v>689420.19100000442</v>
@@ -3602,7 +3598,7 @@
     </row>
     <row r="77" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A77" s="7" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="B77" s="8">
         <v>578064.32600000349</v>
@@ -3623,7 +3619,7 @@
     </row>
     <row r="78" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A78" s="7" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="B78" s="8">
         <v>502291.98900000111</v>
@@ -3644,7 +3640,7 @@
     </row>
     <row r="79" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A79" s="7" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="B79" s="8">
         <v>487107.48900000111</v>
@@ -3665,7 +3661,7 @@
     </row>
     <row r="80" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A80" s="7" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="B80" s="8">
         <v>531998.72900000366</v>
@@ -3686,7 +3682,7 @@
     </row>
     <row r="81" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A81" s="7" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="B81" s="8">
         <v>479733.16099999956</v>
@@ -3707,7 +3703,7 @@
     </row>
     <row r="82" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A82" s="7" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="B82" s="8">
         <v>464263.68299999955</v>
@@ -3728,7 +3724,7 @@
     </row>
     <row r="83" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A83" s="7" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="B83" s="8">
         <v>512991.90999999776</v>
@@ -3749,7 +3745,7 @@
     </row>
     <row r="84" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A84" s="7" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="B84" s="8">
         <v>457884.93900000054</v>
@@ -3770,7 +3766,7 @@
     </row>
     <row r="85" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A85" s="7" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="B85" s="8">
         <v>470890.7450000004</v>
@@ -3791,7 +3787,7 @@
     </row>
     <row r="86" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A86" s="7" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="B86" s="8">
         <v>461411.33</v>
@@ -3812,7 +3808,7 @@
     </row>
     <row r="87" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A87" s="7" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="B87" s="8">
         <v>548439.34500000335</v>
@@ -4016,37 +4012,37 @@
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.15">
       <c r="A1" s="9" t="s">
+        <v>175</v>
+      </c>
+      <c r="B1" s="10" t="s">
         <v>176</v>
       </c>
-      <c r="B1" s="10" t="s">
+      <c r="C1" s="10" t="s">
         <v>177</v>
       </c>
-      <c r="C1" s="10" t="s">
+      <c r="D1" s="10" t="s">
         <v>178</v>
       </c>
-      <c r="D1" s="10" t="s">
+      <c r="E1" s="10" t="s">
         <v>179</v>
       </c>
-      <c r="E1" s="10" t="s">
+      <c r="F1" s="10" t="s">
         <v>180</v>
       </c>
-      <c r="F1" s="10" t="s">
+      <c r="G1" s="10" t="s">
         <v>181</v>
       </c>
-      <c r="G1" s="10" t="s">
+      <c r="H1" s="10" t="s">
         <v>182</v>
       </c>
-      <c r="H1" s="10" t="s">
+      <c r="I1" s="10" t="s">
         <v>183</v>
       </c>
-      <c r="I1" s="10" t="s">
+      <c r="J1" s="10" t="s">
         <v>184</v>
       </c>
-      <c r="J1" s="10" t="s">
+      <c r="K1" s="10" t="s">
         <v>185</v>
-      </c>
-      <c r="K1" s="10" t="s">
-        <v>186</v>
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.15">
@@ -7812,7 +7808,7 @@
         <v>72</v>
       </c>
       <c r="C1" t="s">
-        <v>73</v>
+        <v>190</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.15">
@@ -7910,15 +7906,8 @@
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.15">
-      <c r="A10" t="s">
-        <v>191</v>
-      </c>
-      <c r="B10" s="4">
-        <v>1376120.09</v>
-      </c>
-      <c r="C10" s="5">
-        <v>438625.28000000003</v>
-      </c>
+      <c r="B10" s="4"/>
+      <c r="C10" s="5"/>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.15">
       <c r="B14" s="14"/>
@@ -7942,7 +7931,7 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A1" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B1" s="5" t="s">
         <v>43</v>
@@ -8042,18 +8031,18 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.15">
       <c r="A1" t="s">
+        <v>84</v>
+      </c>
+      <c r="B1" t="s">
+        <v>74</v>
+      </c>
+      <c r="C1" t="s">
         <v>85</v>
-      </c>
-      <c r="B1" t="s">
-        <v>75</v>
-      </c>
-      <c r="C1" t="s">
-        <v>86</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.15">
       <c r="A2" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B2">
         <v>2023</v>
@@ -8064,7 +8053,7 @@
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.15">
       <c r="A3" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B3">
         <v>2023</v>
@@ -8075,7 +8064,7 @@
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.15">
       <c r="A4" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B4">
         <v>2023</v>
@@ -8086,7 +8075,7 @@
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.15">
       <c r="A5" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B5">
         <v>2023</v>
@@ -8097,7 +8086,7 @@
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.15">
       <c r="A6" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B6">
         <v>2023</v>
@@ -8108,7 +8097,7 @@
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.15">
       <c r="A7" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B7">
         <v>2023</v>
@@ -8119,7 +8108,7 @@
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.15">
       <c r="A8" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B8">
         <v>2023</v>
@@ -8130,7 +8119,7 @@
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.15">
       <c r="A9" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B9">
         <v>2023</v>
@@ -8141,7 +8130,7 @@
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.15">
       <c r="A10" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B10">
         <v>2024</v>
@@ -8152,7 +8141,7 @@
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.15">
       <c r="A11" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B11">
         <v>2024</v>
@@ -8163,7 +8152,7 @@
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.15">
       <c r="A12" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B12">
         <v>2024</v>
@@ -8174,7 +8163,7 @@
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.15">
       <c r="A13" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B13">
         <v>2024</v>
@@ -8185,7 +8174,7 @@
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.15">
       <c r="A14" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B14">
         <v>2024</v>
@@ -8196,7 +8185,7 @@
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.15">
       <c r="A15" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B15">
         <v>2024</v>
@@ -8207,7 +8196,7 @@
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.15">
       <c r="A16" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B16">
         <v>2024</v>
@@ -8218,7 +8207,7 @@
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.15">
       <c r="A17" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B17">
         <v>2024</v>
@@ -8229,7 +8218,7 @@
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.15">
       <c r="A18" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B18">
         <v>2025</v>
@@ -8241,7 +8230,7 @@
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.15">
       <c r="A19" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B19">
         <v>2025</v>
@@ -8253,7 +8242,7 @@
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.15">
       <c r="A20" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B20">
         <v>2025</v>
@@ -8265,7 +8254,7 @@
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.15">
       <c r="A21" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B21">
         <v>2025</v>
@@ -8277,7 +8266,7 @@
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.15">
       <c r="A22" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B22">
         <v>2025</v>
@@ -8289,7 +8278,7 @@
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.15">
       <c r="A23" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B23">
         <v>2025</v>
@@ -8300,7 +8289,7 @@
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.15">
       <c r="A24" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B24">
         <v>2025</v>
@@ -8312,7 +8301,7 @@
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.15">
       <c r="A25" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B25">
         <v>2025</v>
@@ -8323,7 +8312,7 @@
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.15">
       <c r="A26" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B26">
         <v>2025</v>
@@ -8335,7 +8324,7 @@
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.15">
       <c r="A27" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B27">
         <v>2026</v>
@@ -8347,7 +8336,7 @@
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.15">
       <c r="A28" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B28">
         <v>2026</v>
@@ -8359,7 +8348,7 @@
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.15">
       <c r="A29" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B29">
         <v>2026</v>
@@ -8371,7 +8360,7 @@
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.15">
       <c r="A30" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B30">
         <v>2026</v>
@@ -8383,7 +8372,7 @@
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.15">
       <c r="A31" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B31">
         <v>2026</v>
@@ -8395,7 +8384,7 @@
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.15">
       <c r="A32" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B32">
         <v>2026</v>
@@ -8406,7 +8395,7 @@
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.15">
       <c r="A33" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B33">
         <v>2026</v>
@@ -8418,7 +8407,7 @@
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.15">
       <c r="A34" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B34">
         <v>2026</v>
@@ -8429,7 +8418,7 @@
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.15">
       <c r="A35" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="B35">
         <v>2026</v>

</xml_diff>

<commit_message>
Auto commit at 2026-05-21  9:19:05.89
</commit_message>
<xml_diff>
--- a/data/homepage.xlsx
+++ b/data/homepage.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" codeName="ThisWorkbook" defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" firstSheet="1" activeTab="6"/>
+    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="Metrics" sheetId="1" r:id="rId1"/>
@@ -1282,7 +1282,7 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="43" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="176" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -1310,15 +1310,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
-    <xf numFmtId="178" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="4" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="181" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1986,7 +1977,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Sheet5"/>
-  <dimension ref="A1:F95"/>
+  <dimension ref="A1:F92"/>
   <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="1" max="1" width="17.125" style="6" customWidth="1"/>
@@ -3913,86 +3904,19 @@
         <v>45993</v>
       </c>
       <c r="B92" s="15">
-        <v>433385.02</v>
+        <v>433163.62</v>
       </c>
       <c r="C92" s="10">
-        <f>234130.17+4226.71</f>
-        <v>238356.88</v>
+        <v>238229.73</v>
       </c>
       <c r="D92" s="15">
-        <f>1856.38+130334.52</f>
-        <v>132190.9</v>
+        <v>132134.94</v>
       </c>
       <c r="E92" s="15">
-        <f>364464.69+6083.09</f>
-        <v>370547.78</v>
+        <v>370364.67</v>
       </c>
       <c r="F92" s="10">
-        <f>17187 +390</f>
-        <v>17577</v>
-      </c>
-    </row>
-    <row r="93" spans="1:6" x14ac:dyDescent="0.15">
-      <c r="A93" s="17">
-        <v>46023</v>
-      </c>
-      <c r="B93" s="18">
-        <v>580496.03</v>
-      </c>
-      <c r="C93" s="18">
-        <v>288277.65999999997</v>
-      </c>
-      <c r="D93" s="18">
-        <v>164409.51999999999</v>
-      </c>
-      <c r="E93" s="18">
-        <v>452687.18</v>
-      </c>
-      <c r="F93" s="18">
-        <v>23473</v>
-      </c>
-    </row>
-    <row r="94" spans="1:6" x14ac:dyDescent="0.15">
-      <c r="A94" s="17">
-        <v>46055</v>
-      </c>
-      <c r="B94" s="18">
-        <v>344816.15</v>
-      </c>
-      <c r="C94" s="18">
-        <f>57206.52+139442.38</f>
-        <v>196648.9</v>
-      </c>
-      <c r="D94" s="19">
-        <v>119481.81</v>
-      </c>
-      <c r="E94" s="19">
-        <f>D94+C94</f>
-        <v>316130.70999999996</v>
-      </c>
-      <c r="F94" s="18">
-        <f>10561+3138</f>
-        <v>13699</v>
-      </c>
-    </row>
-    <row r="95" spans="1:6" x14ac:dyDescent="0.15">
-      <c r="A95" s="17">
-        <v>46084</v>
-      </c>
-      <c r="B95" s="10">
-        <v>450668.16</v>
-      </c>
-      <c r="C95" s="10">
-        <v>231015.32</v>
-      </c>
-      <c r="D95" s="19">
-        <v>154708.91</v>
-      </c>
-      <c r="E95" s="19">
-        <v>385724.23</v>
-      </c>
-      <c r="F95" s="10">
-        <v>18788</v>
+        <v>17570</v>
       </c>
     </row>
   </sheetData>
@@ -7200,16 +7124,16 @@
       <c r="A92" s="9">
         <v>46084</v>
       </c>
-      <c r="B92" s="21">
+      <c r="B92" s="18">
         <v>5759.6</v>
       </c>
-      <c r="C92" s="21">
+      <c r="C92" s="18">
         <v>1603.87</v>
       </c>
-      <c r="D92" s="21">
+      <c r="D92" s="18">
         <v>9252.93</v>
       </c>
-      <c r="E92" s="21">
+      <c r="E92" s="18">
         <v>2200.4</v>
       </c>
       <c r="F92" s="10">
@@ -7391,7 +7315,7 @@
     <row r="1" spans="1:15" x14ac:dyDescent="0.15">
       <c r="A1" s="3">
         <f ca="1">TODAY()-1</f>
-        <v>46142</v>
+        <v>46162</v>
       </c>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.15">
@@ -7428,7 +7352,7 @@
       <c r="A5" t="s">
         <v>44</v>
       </c>
-      <c r="B5" s="20">
+      <c r="B5" s="17">
         <v>20689.639999999996</v>
       </c>
       <c r="C5" t="s">

</xml_diff>